<commit_message>
[auto-transform] rebuild Japan.csv + masterfile.xlsx from master change
</commit_message>
<xml_diff>
--- a/japan-ma/data/masterfile.xlsx
+++ b/japan-ma/data/masterfile.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Japan_Master" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Japan_Master" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -489,292 +477,292 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Deal ID</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Date Announced</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Date Completed / Failed</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Time to Close (months)</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Conclusion / Status</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Target Full Name</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Target Ticker / Exchange</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Industry</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Acquirer Full Name</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Acquirer Listed Exchange</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Deal Size (US$ mn)</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Deal Size (local, JPY bn unless noted)</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>Deal Structure</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>Final Offer Price (local)</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>Initial Offer / Price Bumps</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>Unaffected Price (local)</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>Premium to Unaffected (%)</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>Board Recommendation</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>Special Committee</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>Competing Bid / Interloper</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>Recurring Attempt by Same Acquirer?</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>Toehold / Irrevocables / Tender Agreements</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>Regulator 1</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>Regulator 2</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>Regulator 3</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>Rules / Regulations Triggering Review</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>Key Debate Points / Frictions</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>Activism &amp; Hedge Fund Involvement</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>Final Resolution Mechanism</t>
         </is>
       </c>
-      <c r="AE1" s="1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>Squeeze-out Mechanism</t>
         </is>
       </c>
-      <c r="AF1" s="1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>Delisting Date</t>
         </is>
       </c>
-      <c r="AG1" s="1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>Verification Status</t>
         </is>
       </c>
-      <c r="AH1" s="1" t="inlineStr">
+      <c r="AH1" t="inlineStr">
         <is>
           <t>Notes / Follow-ups</t>
         </is>
       </c>
-      <c r="AI1" s="1" t="inlineStr">
+      <c r="AI1" t="inlineStr">
         <is>
           <t>Source URL 1 (primary)</t>
         </is>
       </c>
-      <c r="AJ1" s="1" t="inlineStr">
+      <c r="AJ1" t="inlineStr">
         <is>
           <t>Source URL 2</t>
         </is>
       </c>
-      <c r="AK1" s="1" t="inlineStr">
+      <c r="AK1" t="inlineStr">
         <is>
           <t>Source URL 3</t>
         </is>
       </c>
-      <c r="AL1" s="1" t="inlineStr">
+      <c r="AL1" t="inlineStr">
         <is>
           <t>Filing / First Report Date</t>
         </is>
       </c>
-      <c r="AM1" s="1" t="inlineStr">
+      <c r="AM1" t="inlineStr">
         <is>
           <t>Pre-Event Close (T-1, local)</t>
         </is>
       </c>
-      <c r="AN1" s="1" t="inlineStr">
+      <c r="AN1" t="inlineStr">
         <is>
           <t>Post-Event Close (T+1, local)</t>
         </is>
       </c>
-      <c r="AO1" s="1" t="inlineStr">
+      <c r="AO1" t="inlineStr">
         <is>
           <t>Premium to T-1 Close (%)</t>
         </is>
       </c>
-      <c r="AP1" s="1" t="inlineStr">
+      <c r="AP1" t="inlineStr">
         <is>
           <t>Market Reaction T+1 (%)</t>
         </is>
       </c>
-      <c r="AQ1" s="1" t="inlineStr">
+      <c r="AQ1" t="inlineStr">
         <is>
           <t>Min Tender Condition (Y/N)</t>
         </is>
       </c>
-      <c r="AR1" s="1" t="inlineStr">
+      <c r="AR1" t="inlineStr">
         <is>
           <t>Min Tender Condition Detail</t>
         </is>
       </c>
-      <c r="AS1" s="1" t="inlineStr">
+      <c r="AS1" t="inlineStr">
         <is>
           <t>Fairness Opinion Provider</t>
         </is>
       </c>
-      <c r="AT1" s="1" t="inlineStr">
+      <c r="AT1" t="inlineStr">
         <is>
           <t>Financial Advisor (Target)</t>
         </is>
       </c>
-      <c r="AU1" s="1" t="inlineStr">
+      <c r="AU1" t="inlineStr">
         <is>
           <t>Financial Advisor (Acquirer)</t>
         </is>
       </c>
-      <c r="AV1" s="1" t="inlineStr">
+      <c r="AV1" t="inlineStr">
         <is>
           <t>Target IPO Lead Underwriter</t>
         </is>
       </c>
-      <c r="AW1" s="1" t="inlineStr">
+      <c r="AW1" t="inlineStr">
         <is>
           <t>FEFTA Classification</t>
         </is>
       </c>
-      <c r="AX1" s="1" t="inlineStr">
+      <c r="AX1" t="inlineStr">
         <is>
           <t>Financing Description</t>
         </is>
       </c>
-      <c r="AY1" s="1" t="inlineStr">
+      <c r="AY1" t="inlineStr">
         <is>
           <t>Break Fee (Y/N)</t>
         </is>
       </c>
-      <c r="AZ1" s="1" t="inlineStr">
+      <c r="AZ1" t="inlineStr">
         <is>
           <t>Break Fee Amount</t>
         </is>
       </c>
-      <c r="BA1" s="1" t="inlineStr">
+      <c r="BA1" t="inlineStr">
         <is>
           <t>TSE Segment</t>
         </is>
       </c>
-      <c r="BB1" s="1" t="inlineStr">
+      <c r="BB1" t="inlineStr">
         <is>
           <t>Index Membership</t>
         </is>
       </c>
-      <c r="BC1" s="1" t="inlineStr">
+      <c r="BC1" t="inlineStr">
         <is>
           <t>Founder/Family Ownership %</t>
         </is>
       </c>
-      <c r="BD1" s="1" t="inlineStr">
+      <c r="BD1" t="inlineStr">
         <is>
           <t>Key Management Age at Announcement</t>
         </is>
       </c>
-      <c r="BE1" s="1" t="inlineStr">
+      <c r="BE1" t="inlineStr">
         <is>
           <t>PBR at Announcement</t>
         </is>
       </c>
-      <c r="BF1" s="1" t="inlineStr">
+      <c r="BF1" t="inlineStr">
         <is>
           <t>date_announced_basis</t>
         </is>

</xml_diff>